<commit_message>
fix: planilha M1 com 47 funcoes unicas (remove duplicata, inclui NtQueryInformationProcess)
</commit_message>
<xml_diff>
--- a/funcoes-mapeadas/fluxos_mapeados.xlsx
+++ b/funcoes-mapeadas/fluxos_mapeados.xlsx
@@ -398,6 +398,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B48"/>
+  <cols>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="110.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -657,106 +661,106 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>QueryPerformanceCounter</v>
+        <v>NtQueryInformationProcess</v>
       </c>
       <c r="B33" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/QueryPerformanceCounter</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/ZwQueryInformationProcess</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>RtlAllocateHeap</v>
+        <v>QueryPerformanceCounter</v>
       </c>
       <c r="B34" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/RtlAllocateHeap</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/QueryPerformanceCounter</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>RtlEncodePointer</v>
+        <v>RtlAllocateHeap</v>
       </c>
       <c r="B35" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/RtlEncodePointer</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/RtlAllocateHeap</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>RtlLeaveCriticalSection</v>
+        <v>RtlEncodePointer</v>
       </c>
       <c r="B36" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/RtlLeaveCriticalSection</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/RtlEncodePointer</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>RtlMoveMemory</v>
+        <v>RtlLeaveCriticalSection</v>
       </c>
       <c r="B37" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/RtlMoveMemory</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/RtlLeaveCriticalSection</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>RtlSizeHeap</v>
+        <v>RtlMoveMemory</v>
       </c>
       <c r="B38" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/RtlSizeHeap</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/RtlMoveMemory</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>SetHandleCount</v>
+        <v>RtlSizeHeap</v>
       </c>
       <c r="B39" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/SetHandleCount</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/RtlSizeHeap</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>SetLastError</v>
+        <v>SetHandleCount</v>
       </c>
       <c r="B40" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/SetLastError</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/SetHandleCount</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>SetUnhandledExceptionFilter</v>
+        <v>SetLastError</v>
       </c>
       <c r="B41" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/SetUnhandledExceptionFilter</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/SetLastError</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>VirtualAlloc</v>
+        <v>SetUnhandledExceptionFilter</v>
       </c>
       <c r="B42" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/VirtualAlloc</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/SetUnhandledExceptionFilter</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>VirtualProtect</v>
+        <v>VirtualAlloc</v>
       </c>
       <c r="B43" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/VirtualProtect</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/VirtualAlloc</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>WaitForSingleObject</v>
+        <v>VirtualProtect</v>
       </c>
       <c r="B44" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/WaitForSingleObject</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/VirtualProtect</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>WideCharToMultiByte</v>
+        <v>WaitForSingleObject</v>
       </c>
       <c r="B45" t="str">
-        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/WideCharToMultiByte</v>
+        <v>https://github.com/fluxtrace/fluxtrace/tree/main/funcoes-mapeadas/WaitForSingleObject</v>
       </c>
     </row>
     <row r="46">

</xml_diff>